<commit_message>
Logging data in files - Update
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="RoutesData" sheetId="1" r:id="rId1"/>
+    <sheet name="RoutesData" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -435,100 +435,85 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{049FB1B4-2A61-4643-8816-8B76EC36FD4B}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="40.69921875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.69921875" style="1" customWidth="1"/>
-  </cols>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1">
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
+      <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C7">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[TTS] Language inititalization + Language setting from UI
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="RoutesData" sheetId="2" r:id="rId5"/>
+    <sheet name="RoutesData" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -435,7 +435,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -453,67 +453,56 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[RFID Reader Integration] Configured CMake and added basic logic
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="RoutesData" sheetId="16" r:id="rId19"/>
+    <sheet name="RoutesData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -435,11 +435,104 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{049FB1B4-2A61-4643-8816-8B76EC36FD4B}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="40.69921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="42.69921875" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Data Collection] Excel Update + UI update
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="RoutesData" sheetId="1" r:id="rId1"/>
+    <sheet name="RoutesData" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -435,101 +435,75 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{049FB1B4-2A61-4643-8816-8B76EC36FD4B}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="40.69921875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="42.69921875" style="1" customWidth="1"/>
-  </cols>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1">
-        <v>20</v>
+      <c r="C4">
+        <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
+    <row r="6">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="C6">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Main Application Integration Updates
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -459,7 +459,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +492,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>32</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TTS Bug fix + Safety Thread Bug Fix
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -459,7 +459,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -470,7 +470,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +481,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -492,7 +492,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -503,7 +503,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Obstacle Avoidance] New impl + Limiting Direction Angle + Bug fixes
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diploma Project - GitLab\diplomaproject\VisionVoyagerGUI\DataCollection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F4567E-9EFE-4F76-AA49-CF6B3656B9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{405262C1-D3CD-4AD7-A09F-2E759E7D157A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="RoutesData" sheetId="3" r:id="rId6"/>
+    <sheet name="RoutesData" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t>Route Name</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Section B</t>
   </si>
   <si>
-    <t>Section C</t>
-  </si>
-  <si>
     <t>Auditorium</t>
   </si>
   <si>
@@ -65,29 +62,15 @@
     <t>Amfiteatrul D1</t>
   </si>
   <si>
-    <t>Secretariat AC</t>
-  </si>
-  <si>
     <t>Secretariat ETC</t>
-  </si>
-  <si>
-    <t>Receptie</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -115,14 +98,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,12 +412,12 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,59 +428,59 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
       <c r="C4">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Line Follower] New implementation updates
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -436,7 +436,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,7 +447,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -458,7 +458,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>9</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -480,7 +480,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Line Follower] New Route Recording Implementation
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -436,7 +436,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,7 +447,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -458,7 +458,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>28</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -480,7 +480,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Main App] TTS race condition fix
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -436,7 +436,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,7 +447,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -458,7 +458,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>40</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -480,7 +480,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[ObstacleAvoiding] Suspend if new obstacle while avoiding
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -436,7 +436,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>48</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,7 +447,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>49</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -458,7 +458,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>50</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -469,7 +469,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -480,7 +480,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>52</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[RoutePlayer] Updates regarding RFID Integration
</commit_message>
<xml_diff>
--- a/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
+++ b/VisionVoyagerGUI/DataCollection/RoutesData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diploma Project - GitLab\diplomaproject\VisionVoyagerGUI\DataCollection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{405262C1-D3CD-4AD7-A09F-2E759E7D157A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF8B868-335D-4820-892C-27547F781A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>Route Name</t>
   </si>
@@ -59,10 +59,16 @@
     <t>Secretariat</t>
   </si>
   <si>
-    <t>Amfiteatrul D1</t>
-  </si>
-  <si>
-    <t>Secretariat ETC</t>
+    <t>B528</t>
+  </si>
+  <si>
+    <t>B527</t>
+  </si>
+  <si>
+    <t>Secretariat AC</t>
+  </si>
+  <si>
+    <t>Section C</t>
   </si>
 </sst>
 </file>
@@ -414,8 +420,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.5" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -436,7 +446,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -447,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="C3">
-        <v>63</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -458,7 +468,7 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>64</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -469,7 +479,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>65</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -480,7 +490,18 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>66</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>